<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-04 Mila dit stop au salon
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-04.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La cabane de coussins</t>
+          <t>Mila dit stop au salon</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>maison, salon, table, plaid, bois, fenêtre, rayon, savon, pli, cachette</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Victorina, maman</t>
+          <t>Mila, Chouchou, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah et Victorina font une cabane de coussins. Le câlin est trop fort. Sarah dit stop, s'éloigne, rejoint maman sous le plaid.</t>
+          <t>Le plaid rouge tient un pli sur la table. Près du pli, un éclat de plaid brille. Mila veut jouer, maintenant. Chouchou ouvre les bras, serre trop. Sourire parti, poitrine, papa accroupi. Stop, recule. Merci vécu. Pli trop vite, bras derrière le tissu. Elle s'arrête, lit l'éclat. Un éclat de plaid tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante. La pluie tape tout doucement. La lampe fait un rond d'or sur le tapis. Un plaid en laine sent le savon. Le thé de maman fume dans la tasse. Tu entends la gouttière, Sarah ? Oui, maman. Ça chante. C'est la pluie qui descend. Les coussins sont empilés comme une colline. En ce moment même, Sarah joue avec Victorina. Elles font une cabane au salon. Victorina ouvre les bras. Elle serre Sarah trop fort. Sarah est gênée. Le câlin est trop près. Son ventre se serre. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Sarah recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Maman est l'adulte sur le canapé. Maman, c'était trop. Tu as dit stop avec ta voix. Bravo, Sarah. Tu as marché jusqu'à moi. Je t'écoute. Tu veux le plaid sur les genoux ? Oui, maman. Sarah pose sa main dans la main de maman. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Victorina range un coussin rouge. Le coussin est loin, maintenant. La gouttière chante encore. Sarah touche le plaid. La laine est un peu rêche. Puis elle devient chaude. On reste sous le plaid un moment ? Oui. C'est chaud. La tasse de maman fume encore. Ça sent le thé sucré.</t>
+          <t>Le plaid rouge tient un pli sur la table. Ça sent le savon, un peu. Ça sent bon, papa. Tu le sens, le savon, Mila ? Oui, papa. Un rayon glisse sur le pli. Il brille, maman. Le plaid est chaud ? Un peu, maman. La cachette va commencer. Le plaid et la table, d'accord ? Oui, maman. Un fil de laine pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La laine est douce contre la peau. Elle pique, maman. Tu la sens, la laine ? Oui. Près du pli, un éclat de plaid brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plaid. Elle vole, maman. Au-dessus du pli ? Oui, au-dessus. Chouchou pose les mains sur le plaid. Le tissu est un peu lourd. On fait la cachette, Chouchou ? Chouchou serre le bord. Le pli tombe un peu. C'est rouge, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le plaid vers la table. Je veux jouer, maintenant ! La cachette, tout de suite. Tu vois Chouchou, Mila ? Oui, papa. Chouchou ouvre les bras. Elle serre Mila trop fort. Les bras collent trop près. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle serre, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat de plaid tremble, puis tient. Chouchou tient Mila contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Mila regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante. La pluie tape tout doucement. La lampe fait un rond d'or sur le tapis. Un plaid en laine sent le savon. Le thé de maman fume dans la tasse. Tu entends la gouttière, Sarah ? Oui, maman. Ça chante. C'est la pluie qui descend. Les coussins sont empilés comme une colline. En ce moment même, Sarah joue avec Victorina. Elles font une cabane au salon. Victorina ouvre les bras. Elle serre Sarah trop fort. Sarah est gênée. Le câlin est trop près. Son ventre se serre. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Sarah recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Maman est l'adulte sur le canapé. Maman, c'était trop. Tu as dit stop avec ta voix. Bravo, Sarah. Tu as marché jusqu'à moi. Je t'écoute. Tu veux le plaid sur les genoux ? Oui, maman. Sarah pose sa main dans la main de maman. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Victorina range un coussin rouge. Le coussin est loin, maintenant. La gouttière chante encore. Sarah touche le plaid. La laine est un peu rêche. Puis elle devient chaude. On reste sous le plaid un moment ? Oui. C'est chaud. La tasse de maman fume encore. Ça sent le thé sucré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plaid rouge tient un pli sur la table. Ça sent le savon, un peu. Ça sent bon, papa. Tu le sens, le savon, Mila ? Oui, papa. Un rayon glisse sur le pli. Il brille, maman. Le plaid est chaud ? Un peu, maman. La cachette va commencer. Le plaid et la table, d'accord ? Oui, maman. Un fil de laine pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La laine est douce contre la peau. Elle pique, maman. Tu la sens, la laine ? Oui. Près du pli, un &lt;emphasis level="moderate"&gt;éclat de plaid&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plaid. Elle vole, maman. Au-dessus du pli ? Oui, au-dessus. Chouchou pose les mains sur le plaid. Le tissu est un peu lourd. On fait la cachette, Chouchou ? Chouchou serre le bord. Le pli tombe un peu. C'est rouge, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le plaid vers la table. Je veux jouer, maintenant ! La cachette, tout de suite. Tu vois Chouchou, Mila ? Oui, papa. Chouchou ouvre les bras. Elle serre Mila trop fort. Les bras collent trop près. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle serre, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat de plaid tremble, puis tient. Chouchou tient Mila contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Mila regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Zélie joue au salon avec Lila. Lila la serre trop fort. Zélie sent sa poitrine coincée. Elle dit : je n'aime pas. C'est trop. Zélie dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Maman est l'adulte sur le canapé. Zélie va vers maman. Elle dit : c'était trop. Maman l'écoute. Zélie pose sa main dans la main de maman. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. [pause]</t>
+          <t>Le plaid rouge tient un pli sur la table. Ça sent le savon, un peu. Ça sent bon, papa. Tu le sens, le savon, Mila ? Oui, papa. Un rayon glisse sur le pli. Il brille, maman. Le plaid est chaud ? Un peu, maman. La cachette va commencer. Le plaid et la table, d'accord ? Oui, maman. Un fil de laine pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La laine est douce contre la peau. Elle pique, maman. Tu la sens, la laine ? Oui. Près du pli, un &lt;emphasis&gt;éclat de plaid&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plaid. Elle vole, maman. Au-dessus du pli ? Oui, au-dessus. Chouchou pose les mains sur le plaid. Le tissu est un peu lourd. On fait la cachette, Chouchou ? Chouchou serre le bord. Le pli tombe un peu. C'est rouge, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le plaid vers la table. Je veux jouer, maintenant ! La cachette, tout de suite. Tu vois Chouchou, Mila ? Oui, papa. Chouchou ouvre les bras. Elle serre Mila trop fort. Les bras collent trop près. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle serre, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat de plaid tremble, puis tient. Chouchou tient Mila contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Mila regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de plaid</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,56 +1326,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_jouer_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La gouttière chante.
-narrateur|La pluie tape tout doucement.
-narrateur|La lampe fait un rond d'or sur le tapis.
-narrateur|Un plaid en laine sent le savon.
-narrateur|Le thé de maman fume dans la tasse.
-maman|Tu entends la gouttière, Sarah ?
-enfant-f|Oui, maman. Ça chante.
-maman|C'est la pluie qui descend.
-narrateur|Les coussins sont empilés comme une colline.
-narrateur|En ce moment même, Sarah joue avec Victorina.
-narrateur|Elles font une cabane au salon.
-narrateur|Victorina ouvre les bras.
-narrateur|Elle serre Sarah trop fort.
-narrateur|Sarah est gênée.
-narrateur|Le câlin est trop près.
-narrateur|Son ventre se serre.
-narrateur|Ses épaules montent.
-enfant-f|Je n'aime pas.
-enfant-f|C'est trop.
-enfant-f|Stop.
-narrateur|Sarah recule d'un pas.
-narrateur|Elle peut s'éloigner.
-narrateur|Elle s'éloigne vers le canapé.
-narrateur|Maman est l'adulte sur le canapé.
-enfant-f|Maman, c'était trop.
-maman|Tu as dit stop avec ta voix.
-maman|Bravo, Sarah.
-maman|Tu as marché jusqu'à moi.
-maman|Je t'écoute.
-maman|Tu veux le plaid sur les genoux ?
+          <t>narrateur|Le plaid rouge tient un pli sur la table.
+narrateur|Ça sent le savon, un peu.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le savon, Mila ?
+enfant-f|Oui, papa.
+narrateur|Un rayon glisse sur le pli.
+enfant-f|Il brille, maman.
+maman|Le plaid est chaud ?
+enfant-f|Un peu, maman.
+maman|La cachette va commencer.
+maman|Le plaid et la table, d'accord ?
 enfant-f|Oui, maman.
-narrateur|Sarah pose sa main dans la main de maman.
-narrateur|Elle souffle.
-narrateur|Ses épaules descendent.
-maman|Dire stop, c'est permis.
-maman|On s'éloigne.
-maman|On va vers un adulte.
-narrateur|Victorina range un coussin rouge.
-narrateur|Le coussin est loin, maintenant.
-narrateur|La gouttière chante encore.
-narrateur|Sarah touche le plaid.
-narrateur|La laine est un peu rêche.
-narrateur|Puis elle devient chaude.
-maman|On reste sous le plaid un moment ?
-enfant-f|Oui. C'est chaud.
-narrateur|La tasse de maman fume encore.
-narrateur|Ça sent le thé sucré.</t>
+narrateur|Un fil de laine pend vers le bois.
+enfant-f|Il pend, papa.
+papa|Tu le vois, le fil ?
+enfant-f|Oui.
+narrateur|La laine est douce contre la peau.
+enfant-f|Elle pique, maman.
+maman|Tu la sens, la laine ?
+enfant-f|Oui.
+narrateur|Près du pli, un éclat de plaid brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Une poussière danse au-dessus du plaid.
+enfant-f|Elle vole, maman.
+maman|Au-dessus du pli ?
+enfant-f|Oui, au-dessus.
+narrateur|Chouchou pose les mains sur le plaid.
+narrateur|Le tissu est un peu lourd.
+enfant-f|On fait la cachette, Chouchou ?
+narrateur|Chouchou serre le bord.
+narrateur|Le pli tombe un peu.
+enfant-f|C'est rouge, papa.
+papa|Comme une maison ?
+enfant-f|Oui, comme une maison.
+narrateur|En ce moment, Mila tire le plaid vers la table.
+enfant-f|Je veux jouer, maintenant !
+enfant-f|La cachette, tout de suite.
+papa|Tu vois Chouchou, Mila ?
+enfant-f|Oui, papa.
+narrateur|Chouchou ouvre les bras.
+narrateur|Elle serre Mila trop fort.
+narrateur|Les bras collent trop près.
+enfant-f|Oh.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules montent un peu.
+papa|Elle serre, Mila ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont serrées, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de plaid tremble, puis tient.
+narrateur|Chouchou tient Mila contre elle.
+enfant-f|C'est trop, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Mila regarde papa.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1407,17 +1421,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Sarah. Que dit-elle ?</t>
+          <t>C'est trop pour Mila. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Sarah. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est trop pour &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Zélie. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est trop pour &lt;emphasis&gt;Mila&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1442,7 +1456,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Zélie dit stop. Puis elle va où ?</t>
+          <t>Mila dit stop. Puis elle va où ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1480,7 +1494,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1491,7 +1505,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1506,34 +1520,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1548,22 +1566,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=cest_trop_pour_mila_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Sarah. Que dit-elle ?</t>
+          <t>narrateur|C'est trop pour Mila.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1609,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a dit stop. Elle a pu s'éloigner. Elle a rejoint maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. Le plaid est chaud sur ses genoux. Le thé fume encore.</t>
+          <t>Mila veut la cachette, tout de suite. Je joue, maintenant ! Elle avance trop vite vers Chouchou. Les bras de Chouchou se referment. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. Stop. Mila recule d'un pas. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le plaid, un instant. Elle écoute le silence du salon. Tu veux la cachette avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, les bras ouverts. Elle recule, plus loin. Chouchou souffle. La cachette. J'aime la cachette. Chouchou pose le plaid sur la table. Merci, Mila. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le pli tient, un peu de travers. La cachette. Elle a un toit, là ? Oui, là. Mila glisse la main près du plaid. La laine est douce, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Chouchou s'assoit, puis se relève. Oui. On le pose au bord ? Le plaid va jusqu'à la table. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a dit stop. Elle a pu s'éloigner. Elle a rejoint maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. Le plaid est chaud sur ses genoux. Le thé fume encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut la cachette, tout de suite. Je joue, maintenant ! Elle avance trop vite vers Chouchou. Les bras de Chouchou se referment. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. &lt;emphasis level="moderate"&gt;Stop&lt;/emphasis&gt;. Mila recule d'un pas. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le plaid, un instant. Elle écoute le silence du salon. Tu veux la cachette avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, les bras ouverts. Elle recule, plus loin. Chouchou souffle. La cachette. J'aime la cachette. Chouchou pose le plaid sur la table. Merci, Mila. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le pli tient, un peu de travers. La cachette. Elle a un toit, là ? Oui, là. Mila glisse la main près du plaid. La laine est douce, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Chouchou s'assoit, puis se relève. Oui. On le pose au bord ? Le plaid va jusqu'à la table. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Zélie a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle a pu s'éloigner. Elle rejoint maman, l'adulte. [pause]</t>
+          <t>Mila veut la cachette, tout de suite. Je joue, maintenant ! Elle avance trop vite vers Chouchou. Les bras de Chouchou se referment. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. &lt;emphasis&gt;Stop&lt;/emphasis&gt;. Mila recule d'un pas. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le plaid, un instant. Elle écoute le silence du salon. Tu veux la cachette avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, les bras ouverts. Elle recule, plus loin. Chouchou souffle. La cachette. J'aime la cachette. Chouchou pose le plaid sur la table. Merci, Mila. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le pli tient, un peu de travers. La cachette. Elle a un toit, là ? Oui, là. Mila glisse la main près du plaid. La laine est douce, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Chouchou s'assoit, puis se relève. Oui. On le pose au bord ? Le plaid va jusqu'à la table. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1647,7 +1666,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1655,10 +1674,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1681,30 +1700,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1713,10 +1732,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1729,20 +1748,52 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=gêne puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_dit_stop_elle_recule; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah a dit stop.
-narrateur|Elle a pu s'éloigner.
-narrateur|Elle a rejoint maman, l'adulte.
-maman|Tu as dit stop.
-maman|Bravo.
-maman|Tu restes près de moi ?
-enfant-f|Oui.
-narrateur|Le plaid est chaud sur ses genoux.
-narrateur|Le thé fume encore.</t>
+          <t>narrateur|Mila veut la cachette, tout de suite.
+enfant-f|Je joue, maintenant !
+narrateur|Elle avance trop vite vers Chouchou.
+narrateur|Les bras de Chouchou se referment.
+narrateur|Mila baisse les yeux.
+narrateur|Sa poitrine est coincée.
+enfant-f|C'est trop.
+enfant-f|Stop.
+narrateur|Mila recule d'un pas.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne parle.
+narrateur|Elle observe le plaid, un instant.
+narrateur|Elle écoute le silence du salon.
+papa|Tu veux la cachette avec Chouchou ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On laisse un peu d'air ?
+enfant-f|D'accord.
+narrateur|Mila reste un moment, les bras ouverts.
+narrateur|Elle recule, plus loin.
+narrateur|Chouchou souffle.
+copine|La cachette.
+enfant-f|J'aime la cachette.
+narrateur|Chouchou pose le plaid sur la table.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux, au salon.
+maman|Le tissu est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Le pli tient, un peu de travers.
+enfant-f|La cachette.
+papa|Elle a un toit, là ?
+enfant-f|Oui, là.
+narrateur|Mila glisse la main près du plaid.
+narrateur|La laine est douce, contre la peau.
+maman|Tes mains sont au chaud, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Chouchou s'assoit, puis se relève.
+copine|Oui.
+enfant-f|On le pose au bord ?
+maman|Le plaid va jusqu'à la table.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah reste près du canapé. Maman lui parle tout bas. Ton ventre s'est serré. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. La pluie tapote encore la gouttière. Le rond d'or est toujours sur le tapis. Sarah souffle une dernière fois. Victorina tourne une page d'un livre. Le livre est loin du canapé. Victorina lit là-bas. Toi, tu es ici.</t>
+          <t>Ils restent près de la table. Le plaid tombe d'un côté. Le toit, maintenant ! Mila tire le plaid trop vite. Le pli cache son visage. Je ne vois plus ! Chouchou ouvre les bras, derrière le tissu. Elle serre trop fort, cette fois. Stop ! Mila recule d'un pas, sous le plaid. Chouchou serre les lèvres. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila recule, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le pli, un instant. Elle écoute le silence du salon. Au bord du pli, un éclat de plaid luit. Là, sur le plaid. Tu veux la cachette, Chouchou ? Chouchou ne serre plus. Elle tend les mains, sans coller. Je veux la cachette. Mila tire le plaid, sans se presser. Chouchou le reçoit, plus loin. Le tissu est lisse et tiède. Tu le vois, le pli ? Oui, papa. La cachette est près de la table ? Oui, maman. Chouchou pose un bord. Mila pose une main sur le bois. Le pli tient, Mila ? Oui, papa. Un rayon passe sur le plaid. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah reste près du canapé. Maman lui parle tout bas. Ton ventre s'est serré. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. La pluie tapote encore la gouttière. Le rond d'or est toujours sur le tapis. Sarah souffle une dernière fois. Victorina tourne une page d'un livre. Le livre est loin du canapé. Victorina lit là-bas. Toi, tu es ici.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de la table. Le plaid tombe d'un côté. Le toit, maintenant ! Mila tire le plaid trop vite. Le pli cache son visage. Je ne vois plus ! Chouchou ouvre les bras, derrière le tissu. Elle serre trop fort, cette fois. Stop ! Mila recule d'un pas, sous le plaid. Chouchou serre les lèvres. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila recule, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le pli, un instant. Elle écoute le silence du salon. Au bord du pli, un &lt;emphasis level="moderate"&gt;éclat de plaid&lt;/emphasis&gt; luit. Là, sur le plaid. Tu veux la cachette, Chouchou ? Chouchou ne serre plus. Elle tend les mains, sans coller. Je veux la cachette. Mila tire le plaid, sans se presser. Chouchou le reçoit, plus loin. Le tissu est lisse et tiède. Tu le vois, le pli ? Oui, papa. La cachette est près de la table ? Oui, maman. Chouchou pose un bord. Mila pose une main sur le bois. Le pli tient, Mila ? Oui, papa. Un rayon passe sur le plaid. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Zélie reste près du canapé. Maman lui parle tout bas. [pause]</t>
+          <t>Ils restent près de la table. Le plaid tombe d'un côté. Le toit, maintenant ! Mila tire le plaid trop vite. Le pli cache son visage. Je ne vois plus ! Chouchou ouvre les bras, derrière le tissu. Elle serre trop fort, cette fois. Stop ! Mila recule d'un pas, sous le plaid. Chouchou serre les lèvres. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila recule, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le pli, un instant. Elle écoute le silence du salon. Au bord du pli, un &lt;emphasis&gt;éclat de plaid&lt;/emphasis&gt; luit. Là, sur le plaid. Tu veux la cachette, Chouchou ? Chouchou ne serre plus. Elle tend les mains, sans coller. Je veux la cachette. Mila tire le plaid, sans se presser. Chouchou le reçoit, plus loin. Le tissu est lisse et tiède. Tu le vois, le pli ? Oui, papa. La cachette est près de la table ? Oui, maman. Chouchou pose un bord. Mila pose une main sur le bois. Le pli tient, Mila ? Oui, papa. Un rayon passe sur le plaid. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1826,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1834,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1858,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plaid</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,22 +1957,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=pli_trop_vite_bras_derriere_elle_recule; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah reste près du canapé.
-narrateur|Maman lui parle tout bas.
-maman|Ton ventre s'est serré.
-maman|Tu as écouté.
-maman|Tu es plus calme, maintenant ?
+          <t>narrateur|Ils restent près de la table.
+narrateur|Le plaid tombe d'un côté.
+enfant-f|Le toit, maintenant !
+narrateur|Mila tire le plaid trop vite.
+narrateur|Le pli cache son visage.
+enfant-f|Je ne vois plus !
+narrateur|Chouchou ouvre les bras, derrière le tissu.
+narrateur|Elle serre trop fort, cette fois.
+enfant-f|Stop !
+narrateur|Mila recule d'un pas, sous le plaid.
+narrateur|Chouchou serre les lèvres.
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila recule, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le pli, un instant.
+narrateur|Elle écoute le silence du salon.
+narrateur|Au bord du pli, un éclat de plaid luit.
+enfant-f|Là, sur le plaid.
+enfant-f|Tu veux la cachette, Chouchou ?
+narrateur|Chouchou ne serre plus.
+narrateur|Elle tend les mains, sans coller.
+copine|Je veux la cachette.
+narrateur|Mila tire le plaid, sans se presser.
+narrateur|Chouchou le reçoit, plus loin.
+narrateur|Le tissu est lisse et tiède.
+papa|Tu le vois, le pli ?
+enfant-f|Oui, papa.
+maman|La cachette est près de la table ?
 enfant-f|Oui, maman.
-narrateur|La pluie tapote encore la gouttière.
-narrateur|Le rond d'or est toujours sur le tapis.
-narrateur|Sarah souffle une dernière fois.
-narrateur|Victorina tourne une page d'un livre.
-narrateur|Le livre est loin du canapé.
-maman|Victorina lit là-bas.
-maman|Toi, tu es ici.</t>
+narrateur|Chouchou pose un bord.
+narrateur|Mila pose une main sur le bois.
+papa|Le pli tient, Mila ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le plaid.
+enfant-f|Il allume le bois.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1949,17 +2032,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers maman. Bravo.</t>
+          <t>Ils restent près de la table. La cachette est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le plaid sent le savon. Tu le sens, le savon ? Oui, maman. Le pli reste un peu, de travers. Il a tenu, sur la table. La cachette. Le plaid est chaud, sous les mains. Le pli rouge fait de l'ombre. On y retourne, après. Un éclat de plaid tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers maman. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. La cachette est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le plaid sent le savon. Tu le sens, le savon ? Oui, maman. Le pli reste un peu, de travers. Il a tenu, sur la table. La cachette. Le plaid est chaud, sous les mains. Le pli rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de plaid&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. La cachette est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le plaid sent le savon. Tu le sens, le savon ? Oui, maman. Le pli reste un peu, de travers. Il a tenu, sur la table. La cachette. Le plaid est chaud, sous les mains. Le pli rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de plaid&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,7 +2089,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2014,10 +2097,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2026,12 +2109,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,17 +2123,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plaid</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2059,11 +2146,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,27 +2159,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit stop.
-enfant-f|Je me suis éloignée.
-enfant-f|Je suis allée vers maman.
-maman|Bravo.</t>
+          <t>narrateur|Ils restent près de la table.
+maman|La cachette est arrivée, Mila ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Mila souffle, un filet d'air.
+enfant-f|Le plaid sent le savon.
+maman|Tu le sens, le savon ?
+enfant-f|Oui, maman.
+papa|Le pli reste un peu, de travers.
+enfant-f|Il a tenu, sur la table.
+copine|La cachette.
+narrateur|Le plaid est chaud, sous les mains.
+narrateur|Le pli rouge fait de l'ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat de plaid tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2273,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>